<commit_message>
Génère les fichiers de review de la semaine
À déposer dans le dossier Drive permanent de chaque client (routine Claude du vendredi), qui note leur identifiant dans reviews/config.json.
</commit_message>
<xml_diff>
--- a/reviews/a-envoyer/la-galerie-immobiliere-2026-08-31.xlsx
+++ b/reviews/a-envoyer/la-galerie-immobiliere-2026-08-31.xlsx
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -825,7 +825,7 @@
       <c r="H4" s="10" t="inlineStr"/>
       <c r="I4" s="9" t="inlineStr"/>
     </row>
-    <row r="5" ht="210" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>LGI-04</t>
@@ -838,25 +838,64 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>FB + IG</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>voir le visuel</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Story mercredi 02/09 — Estimation en ligne vs estimation sur place (banque · story-projet · renvoi carrousel 18h)</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr"/>
+      <c r="I5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="210" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>LGI-05</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Mer 02/09</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Carrousel (8 visuels)</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>FB + IG</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>voir le visuel</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Vous avez fait une estimation en ligne et obtenu une fourchette de plusieurs dizaines de milliers d'euros. Normal : un algorithme connaît votre quartier, pas votre bien.
 Voici ce que nous regardons en plus, sur place. Faites défiler.
@@ -865,41 +904,119 @@
 #estimation #immobilierparis #hautsdeseine #vendresonbien #immobilierprestige #copropriete</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr"/>
-      <c r="I5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6" ht="156" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>LGI-05</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>LGI-06</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Jeu 03/09</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>FB + IG</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>voir le visuel</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Story jeudi 03/09 — La lumière, ce critère qu'on sous-estime (banque · story-lumiere)</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>LGI-07</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Ven 04/09</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>FB + IG</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>voir le visuel</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Story vendredi 04/09 — 5 tendances du marché à Puteaux (banque · story-lundi · renvoi post 12h30)</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9" ht="156" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LGI-08</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Ven 04/09</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>FB + IG</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>voir le visuel</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Rentrée 2026 — 5 tendances du marché à Puteaux 📊
 Ce qu'il faut savoir pour bien démarrer son projet immo cette rentrée.
@@ -907,51 +1024,90 @@
 #GalerieImmobiliere #Puteaux #ImmobilierPuteaux #AgenceImmoPuteaux #ConseilImmo #AcheterMaison #VendreSonBien #EstimationGratuite</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="21" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>LGI-06</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10" ht="21" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>LGI-09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Sam 05/09</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Post</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>FB + IG</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>voir le visuel</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>Story samedi 05/09 — Week-end de visites</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>LGI-10</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Dim 06/09</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>FB + IG</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>voir le visuel</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Story dimanche 06/09 — Inspiration du dimanche (banque · story-dimanche)</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <conditionalFormatting sqref="A2:I7">
+  <conditionalFormatting sqref="A2:I11">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$H2="✅ OK pour publier"</formula>
     </cfRule>
@@ -963,7 +1119,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choisir dans la liste" error="Choisissez une des trois décisions du menu, ou laissez la case vide." type="list">
+    <dataValidation sqref="H2:H11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choisir dans la liste" error="Choisissez une des trois décisions du menu, ou laissez la case vide." type="list">
       <formula1>"✅ OK pour publier,✏️ À corriger (voir commentaire),⛔ Ne pas publier"</formula1>
     </dataValidation>
   </dataValidations>
@@ -973,6 +1129,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -984,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1019,7 +1179,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-28T06:09:04</t>
+          <t>2026-08-28T17:14:08</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1217,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>364997930</v>
+        <v>367901967</v>
       </c>
       <c r="C6" t="n">
         <v>5733302</v>
@@ -1080,7 +1240,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>364997942</v>
+        <v>367901978</v>
       </c>
       <c r="C7" t="n">
         <v>5733302</v>
@@ -1129,17 +1289,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>358747927</v>
+        <v>367901986</v>
       </c>
       <c r="C9" t="n">
         <v>5733302</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>2026-09-02T10:00:00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Story mercredi 02/09 — Estimation en ligne vs estimation sur place (banque · story-projet · renvoi carrousel 18h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LGI-05</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>358747927</v>
+      </c>
+      <c r="C10" t="n">
+        <v>5733302</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>2026-09-02T18:00:00</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Vous avez fait une estimation en ligne et obtenu une fourchette de plusieurs dizaines de milliers d'euros. Normal : un algorithme connaît votre quartier, pas votre bien.
 Voici ce que nous regardons en plus, sur place. Faites défiler.
@@ -1149,24 +1332,70 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>LGI-05</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LGI-06</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>367902002</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5733302</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-09-03T10:00:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Story jeudi 03/09 — La lumière, ce critère qu'on sous-estime (banque · story-lumiere)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LGI-07</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>367902009</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5733302</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-09-04T10:00:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Story vendredi 04/09 — 5 tendances du marché à Puteaux (banque · story-lundi · renvoi post 12h30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LGI-08</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>351958196</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C13" t="n">
         <v>5733302</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>2026-09-04T12:30:00</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Rentrée 2026 — 5 tendances du marché à Puteaux 📊
 Ce qu'il faut savoir pour bien démarrer son projet immo cette rentrée.
@@ -1175,26 +1404,49 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LGI-06</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>364997955</v>
-      </c>
-      <c r="C11" t="n">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LGI-09</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>367902022</v>
+      </c>
+      <c r="C14" t="n">
         <v>5733302</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>2026-09-05T10:00:00</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Story samedi 05/09 — Week-end de visites</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LGI-10</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>367902029</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5733302</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-09-06T10:00:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Story dimanche 06/09 — Inspiration du dimanche (banque · story-dimanche)</t>
         </is>
       </c>
     </row>

</xml_diff>